<commit_message>
fix(materials): provide CE a format-only handoff workbook
</commit_message>
<xml_diff>
--- a/public/material-upload-template.xlsx
+++ b/public/material-upload-template.xlsx
@@ -2,8 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上傳資料" sheetId="1" r:id="Ra3027fe167de48a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="2" r:id="Rc355b70a16d04a16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上傳資料" sheetId="1" r:id="R3e7c563ac3fa4ea7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +18,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="General"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -44,12 +43,6 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF242B33"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -160,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -289,48 +282,6 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -560,7 +511,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>CE BOM 空白交付範本</x:v>
+        <x:v>CE BOM 交付格式</x:v>
       </x:c>
       <x:c r="B1" s="6"/>
       <x:c r="C1" s="6"/>
@@ -583,7 +534,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>規格日期 2026-10-21。第 4 列為固定表頭，第 5 列起填資料；請先閱讀「分工與欄位說明」。</x:v>
+        <x:v>第4列表頭請保留，第5列起填寫資料</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -604,77 +555,26 @@
       <x:c r="R2" s="3"/>
       <x:c r="S2" s="3"/>
     </x:row>
-    <x:row r="3" ht="36" customHeight="1">
-      <x:c r="A3" s="11" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
-      </x:c>
-      <x:c r="B3" s="11" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
-      </x:c>
-      <x:c r="C3" s="11" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
-      </x:c>
-      <x:c r="D3" s="11" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
-      </x:c>
-      <x:c r="E3" s="11" t="str">
-        <x:v>RD 提供
-CE 核對</x:v>
-      </x:c>
-      <x:c r="F3" s="11" t="str">
-        <x:v>CE 保留舊格式</x:v>
-      </x:c>
-      <x:c r="G3" s="11" t="str">
-        <x:v>CE 核對
-帶出</x:v>
-      </x:c>
-      <x:c r="H3" s="11" t="str">
-        <x:v>CE 從來源帶出</x:v>
-      </x:c>
-      <x:c r="I3" s="11" t="str">
-        <x:v>CE 從來源帶出</x:v>
-      </x:c>
-      <x:c r="J3" s="11" t="str">
-        <x:v>CE 從來源帶出</x:v>
-      </x:c>
-      <x:c r="K3" s="11" t="str">
-        <x:v>原始分組
-CE 保留</x:v>
-      </x:c>
-      <x:c r="L3" s="11" t="str">
-        <x:v>來源資料
-CE 保留</x:v>
-      </x:c>
-      <x:c r="M3" s="11" t="str">
-        <x:v>來源參考
-CE 保留</x:v>
-      </x:c>
-      <x:c r="N3" s="11" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="O3" s="11" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="P3" s="11" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
-      </x:c>
-      <x:c r="Q3" s="11" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
-      </x:c>
-      <x:c r="R3" s="11" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
-      </x:c>
-      <x:c r="S3" s="12" t="str">
-        <x:v>CE 補欄
-帶出原文</x:v>
-      </x:c>
+    <x:row r="3" ht="10" customHeight="1">
+      <x:c r="A3" s="1"/>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+      <x:c r="I3" s="1"/>
+      <x:c r="J3" s="1"/>
+      <x:c r="K3" s="1"/>
+      <x:c r="L3" s="1"/>
+      <x:c r="M3" s="1"/>
+      <x:c r="N3" s="1"/>
+      <x:c r="O3" s="1"/>
+      <x:c r="P3" s="1"/>
+      <x:c r="Q3" s="1"/>
+      <x:c r="R3" s="1"/>
+      <x:c r="S3" s="1"/>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="21" t="str">
@@ -1368,620 +1268,4 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetPr>
-    <x:tabColor rgb="FF888D93"/>
-  </x:sheetPr>
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="76" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="27" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>CE BOM 交付分工與欄位說明</x:v>
-      </x:c>
-      <x:c r="B1" s="6"/>
-      <x:c r="C1" s="6"/>
-      <x:c r="D1" s="6"/>
-      <x:c r="E1" s="6"/>
-    </x:row>
-    <x:row r="2" ht="25" customHeight="1">
-      <x:c r="A2" s="7" t="str">
-        <x:v>規格日期 2026-10-21</x:v>
-      </x:c>
-      <x:c r="B2" s="3"/>
-      <x:c r="C2" s="3"/>
-      <x:c r="D2" s="3"/>
-      <x:c r="E2" s="3"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="3"/>
-      <x:c r="B3" s="3"/>
-      <x:c r="C3" s="3"/>
-      <x:c r="D3" s="3"/>
-      <x:c r="E3" s="3"/>
-    </x:row>
-    <x:row r="4" ht="27" customHeight="1">
-      <x:c r="A4" s="45" t="str">
-        <x:v>一、作業分工</x:v>
-      </x:c>
-      <x:c r="B4" s="8"/>
-      <x:c r="C4" s="8"/>
-      <x:c r="D4" s="8"/>
-      <x:c r="E4" s="8"/>
-    </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="21" t="str">
-        <x:v>角色</x:v>
-      </x:c>
-      <x:c r="B5" s="22" t="str">
-        <x:v>交付結果</x:v>
-      </x:c>
-      <x:c r="C5" s="23" t="str">
-        <x:v>責任</x:v>
-      </x:c>
-      <x:c r="D5" s="3"/>
-      <x:c r="E5" s="3"/>
-    </x:row>
-    <x:row r="6" ht="48" customHeight="1">
-      <x:c r="A6" s="47" t="str">
-        <x:v>公司現有系統</x:v>
-      </x:c>
-      <x:c r="B6" s="47" t="str">
-        <x:v>公司料號與來源狀態</x:v>
-      </x:c>
-      <x:c r="C6" s="47" t="str">
-        <x:v>維持原本的料號、料況與申請／核准流程，是正式資料來源；本工具不要求修改公司系統。</x:v>
-      </x:c>
-      <x:c r="D6" s="3"/>
-      <x:c r="E6" s="3"/>
-    </x:row>
-    <x:row r="7" ht="48" customHeight="1">
-      <x:c r="A7" s="47" t="str">
-        <x:v>CE</x:v>
-      </x:c>
-      <x:c r="B7" s="47" t="str">
-        <x:v>整理後 BOM＋零件狀態</x:v>
-      </x:c>
-      <x:c r="C7" s="47" t="str">
-        <x:v>依 RD 提供的客戶 BOM，利用公司現有系統整理並轉出清單；保留設計欄位，補上右側「零件狀態」，再交回 RD。查無料號或狀態不明時明確註記待確認。</x:v>
-      </x:c>
-      <x:c r="D7" s="3"/>
-      <x:c r="E7" s="3"/>
-    </x:row>
-    <x:row r="8" ht="48" customHeight="1">
-      <x:c r="A8" s="47" t="str">
-        <x:v>料號追蹤工具</x:v>
-      </x:c>
-      <x:c r="B8" s="47" t="str">
-        <x:v>可檢查的料號總表與追蹤紀錄</x:v>
-      </x:c>
-      <x:c r="C8" s="47" t="str">
-        <x:v>自動讀取欄位、整理主料與替代料、對應 TX、呈現料號與風險；保留原文，不代替公司系統核准料號，也不替 RD 決定能否採用。</x:v>
-      </x:c>
-      <x:c r="D8" s="3"/>
-      <x:c r="E8" s="3"/>
-    </x:row>
-    <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="47" t="str">
-        <x:v>RD</x:v>
-      </x:c>
-      <x:c r="B9" s="47" t="str">
-        <x:v>確認結果與後續申請追蹤</x:v>
-      </x:c>
-      <x:c r="C9" s="47" t="str">
-        <x:v>提供設計 BOM，匯入 CE 清單後核對位號、用量、料號與零件狀態；依公司流程確認選用／申請事項，再於網站記錄追蹤說明、單號與更新人。</x:v>
-      </x:c>
-      <x:c r="D9" s="3"/>
-      <x:c r="E9" s="3"/>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="3"/>
-      <x:c r="B10" s="3"/>
-      <x:c r="C10" s="3"/>
-      <x:c r="D10" s="3"/>
-      <x:c r="E10" s="3"/>
-    </x:row>
-    <x:row r="11" ht="27" customHeight="1">
-      <x:c r="A11" s="45" t="str">
-        <x:v>二、共同規則</x:v>
-      </x:c>
-      <x:c r="B11" s="8"/>
-      <x:c r="C11" s="8"/>
-      <x:c r="D11" s="8"/>
-      <x:c r="E11" s="8"/>
-    </x:row>
-    <x:row r="12" ht="44" customHeight="1">
-      <x:c r="A12" s="48" t="str">
-        <x:v>規則 1</x:v>
-      </x:c>
-      <x:c r="B12" s="48"/>
-      <x:c r="C12" s="47" t="str">
-        <x:v>CE 整理與帶出狀態，不代表 CE 有權變更所有來源狀態；禁用、EOL、ODM 不建議用料等設定仍依公司既有權責窗口處理。</x:v>
-      </x:c>
-      <x:c r="D12" s="48"/>
-      <x:c r="E12" s="48"/>
-    </x:row>
-    <x:row r="13" ht="44" customHeight="1">
-      <x:c r="A13" s="48" t="str">
-        <x:v>規則 2</x:v>
-      </x:c>
-      <x:c r="B13" s="48"/>
-      <x:c r="C13" s="47" t="str">
-        <x:v>Sourcing Status 是供應／核准來源狀態；零件狀態是新設計使用限制。兩欄分開保留。Approved／Active 不代表可以忽略禁用或 ODM 不建議用料。</x:v>
-      </x:c>
-      <x:c r="D13" s="48"/>
-      <x:c r="E13" s="48"/>
-    </x:row>
-    <x:row r="14" ht="44" customHeight="1">
-      <x:c r="A14" s="48" t="str">
-        <x:v>規則 3</x:v>
-      </x:c>
-      <x:c r="B14" s="48"/>
-      <x:c r="C14" s="47" t="str">
-        <x:v>零件狀態放在 BOM 最右側，由 CE 帶出公司原文；未確認時填待確認，不得自行改填 Approved 或可用。查無公司料號時，Part Number 保持空白。</x:v>
-      </x:c>
-      <x:c r="D14" s="48"/>
-      <x:c r="E14" s="48"/>
-    </x:row>
-    <x:row r="15" ht="44" customHeight="1">
-      <x:c r="A15" s="48" t="str">
-        <x:v>規則 4</x:v>
-      </x:c>
-      <x:c r="B15" s="48"/>
-      <x:c r="C15" s="47" t="str">
-        <x:v>料號追蹤、單號、EE 是 RD 在網站維護的作業紀錄，CE 不需為了交付清單額外填寫；零件狀態不會自動建立申請追蹤。</x:v>
-      </x:c>
-      <x:c r="D15" s="48"/>
-      <x:c r="E15" s="48"/>
-    </x:row>
-    <x:row r="16" ht="44" customHeight="1">
-      <x:c r="A16" s="48" t="str">
-        <x:v>規則 5</x:v>
-      </x:c>
-      <x:c r="B16" s="48"/>
-      <x:c r="C16" s="47" t="str">
-        <x:v>範例中的料號、廠商與狀態都是格式示範，不能當成真實選料、核准或替代料相容性依據。</x:v>
-      </x:c>
-      <x:c r="D16" s="48"/>
-      <x:c r="E16" s="48"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="3"/>
-      <x:c r="B17" s="3"/>
-      <x:c r="C17" s="3"/>
-      <x:c r="D17" s="3"/>
-      <x:c r="E17" s="3"/>
-    </x:row>
-    <x:row r="18" ht="27" customHeight="1">
-      <x:c r="A18" s="45" t="str">
-        <x:v>三、交付與匯入步驟</x:v>
-      </x:c>
-      <x:c r="B18" s="8"/>
-      <x:c r="C18" s="8"/>
-      <x:c r="D18" s="8"/>
-      <x:c r="E18" s="8"/>
-    </x:row>
-    <x:row r="19" ht="44" customHeight="1">
-      <x:c r="A19" s="48" t="str">
-        <x:v>步驟 1</x:v>
-      </x:c>
-      <x:c r="B19" s="48"/>
-      <x:c r="C19" s="47" t="str">
-        <x:v>RD 提供單一專案／版本的客戶 BOM，CE 保留設計料名、位號、用量與圖面資料。</x:v>
-      </x:c>
-      <x:c r="D19" s="48"/>
-      <x:c r="E19" s="48"/>
-    </x:row>
-    <x:row r="20" ht="44" customHeight="1">
-      <x:c r="A20" s="48" t="str">
-        <x:v>步驟 2</x:v>
-      </x:c>
-      <x:c r="B20" s="48"/>
-      <x:c r="C20" s="47" t="str">
-        <x:v>CE 利用公司現有系統核對並帶出公司料號、供應狀態等資料，在最右側補上零件狀態；未知處明確填待確認。</x:v>
-      </x:c>
-      <x:c r="D20" s="48"/>
-      <x:c r="E20" s="48"/>
-    </x:row>
-    <x:row r="21" ht="44" customHeight="1">
-      <x:c r="A21" s="48" t="str">
-        <x:v>步驟 3</x:v>
-      </x:c>
-      <x:c r="B21" s="48"/>
-      <x:c r="C21" s="47" t="str">
-        <x:v>CE 依空白範本的固定表頭交付 Excel；一列一個廠商料，同組替代料相鄰排列，保留 Ref_tmp／Ref Des。</x:v>
-      </x:c>
-      <x:c r="D21" s="48"/>
-      <x:c r="E21" s="48"/>
-    </x:row>
-    <x:row r="22" ht="44" customHeight="1">
-      <x:c r="A22" s="48" t="str">
-        <x:v>步驟 4</x:v>
-      </x:c>
-      <x:c r="B22" s="48"/>
-      <x:c r="C22" s="47" t="str">
-        <x:v>RD 使用上傳 BOM 匯入，核對群組數、位號、MPN、公司料號、供應狀態與零件狀態。工具只整理與提示，不自動核准。</x:v>
-      </x:c>
-      <x:c r="D22" s="48"/>
-      <x:c r="E22" s="48"/>
-    </x:row>
-    <x:row r="23" ht="44" customHeight="1">
-      <x:c r="A23" s="48" t="str">
-        <x:v>步驟 5</x:v>
-      </x:c>
-      <x:c r="B23" s="48"/>
-      <x:c r="C23" s="47" t="str">
-        <x:v>RD 依公司流程處理選用與申請；料號追蹤、單號、EE 與圖片於網站維護，再匯出結果供確認。</x:v>
-      </x:c>
-      <x:c r="D23" s="48"/>
-      <x:c r="E23" s="48"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="3"/>
-      <x:c r="B24" s="3"/>
-      <x:c r="C24" s="3"/>
-      <x:c r="D24" s="3"/>
-      <x:c r="E24" s="3"/>
-    </x:row>
-    <x:row r="25" ht="27" customHeight="1">
-      <x:c r="A25" s="45" t="str">
-        <x:v>四、固定欄位與責任</x:v>
-      </x:c>
-      <x:c r="B25" s="8"/>
-      <x:c r="C25" s="8"/>
-      <x:c r="D25" s="8"/>
-      <x:c r="E25" s="8"/>
-    </x:row>
-    <x:row r="26" ht="35" customHeight="1">
-      <x:c r="A26" s="21" t="str">
-        <x:v>Excel 表頭（第 4 列）</x:v>
-      </x:c>
-      <x:c r="B26" s="22" t="str">
-        <x:v>欄位責任</x:v>
-      </x:c>
-      <x:c r="C26" s="22" t="str">
-        <x:v>填寫要求</x:v>
-      </x:c>
-      <x:c r="D26" s="22" t="str">
-        <x:v>匯入位置</x:v>
-      </x:c>
-      <x:c r="E26" s="23" t="str">
-        <x:v>格式示例（DEMO）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="34" customHeight="1">
-      <x:c r="A27" s="50" t="str">
-        <x:v>Level</x:v>
-      </x:c>
-      <x:c r="B27" s="50" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C27" s="51" t="str">
-        <x:v>料件列填 2；0 為系統、1 為模組，網站只建立 Level 2 料件。</x:v>
-      </x:c>
-      <x:c r="D27" s="51" t="str">
-        <x:v>階層／分組</x:v>
-      </x:c>
-      <x:c r="E27" s="56" t="str">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="34" customHeight="1">
-      <x:c r="A28" s="52" t="str">
-        <x:v>Name</x:v>
-      </x:c>
-      <x:c r="B28" s="52" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C28" s="53" t="str">
-        <x:v>保留客戶 BOM 料名；每個料件列必填，不要以廠商名稱取代。</x:v>
-      </x:c>
-      <x:c r="D28" s="53" t="str">
-        <x:v>料件名稱</x:v>
-      </x:c>
-      <x:c r="E28" s="57" t="str">
-        <x:v>CAP CER 0.1UF 16V X7R</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="34" customHeight="1">
-      <x:c r="A29" s="52" t="str">
-        <x:v>Qty</x:v>
-      </x:c>
-      <x:c r="B29" s="52" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C29" s="53" t="str">
-        <x:v>保留設計用量；不要因展開替代料而重算或加總用量。</x:v>
-      </x:c>
-      <x:c r="D29" s="53" t="str">
-        <x:v>數量</x:v>
-      </x:c>
-      <x:c r="E29" s="57" t="str">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="34" customHeight="1">
-      <x:c r="A30" s="52" t="str">
-        <x:v>Ref Des</x:v>
-      </x:c>
-      <x:c r="B30" s="52" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C30" s="53" t="str">
-        <x:v>保留完整位號，逗號分隔；同組替代料使用相同位號。</x:v>
-      </x:c>
-      <x:c r="D30" s="53" t="str">
-        <x:v>REF DES</x:v>
-      </x:c>
-      <x:c r="E30" s="57" t="str">
-        <x:v>C101, C102</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="34" customHeight="1">
-      <x:c r="A31" s="52" t="str">
-        <x:v>Manufacturer Part Number(1)</x:v>
-      </x:c>
-      <x:c r="B31" s="52" t="str">
-        <x:v>RD 提供／CE 核對</x:v>
-      </x:c>
-      <x:c r="C31" s="53" t="str">
-        <x:v>每列一個廠商料號；依原 BOM 與公司資料核對，不自行換成未確認替代料。</x:v>
-      </x:c>
-      <x:c r="D31" s="53" t="str">
-        <x:v>MPN</x:v>
-      </x:c>
-      <x:c r="E31" s="57" t="str">
-        <x:v>DEMO-CAP-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="34" customHeight="1">
-      <x:c r="A32" s="52" t="str">
-        <x:v>Manufacturer Part Number(2)</x:v>
-      </x:c>
-      <x:c r="B32" s="52" t="str">
-        <x:v>CE 保留舊格式</x:v>
-      </x:c>
-      <x:c r="C32" s="53" t="str">
-        <x:v>舊格式相容欄，可留白；新交付的其他候選料請各自另列。</x:v>
-      </x:c>
-      <x:c r="D32" s="53" t="str">
-        <x:v>第二 MPN（相容欄）</x:v>
-      </x:c>
-      <x:c r="E32" s="57" t="str">
-        <x:v>留白</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="34" customHeight="1">
-      <x:c r="A33" s="52" t="str">
-        <x:v>Manufacturer</x:v>
-      </x:c>
-      <x:c r="B33" s="52" t="str">
-        <x:v>CE 核對／帶出</x:v>
-      </x:c>
-      <x:c r="C33" s="53" t="str">
-        <x:v>填該列 MPN 對應的廠商，不把不同廠商合在同一列。</x:v>
-      </x:c>
-      <x:c r="D33" s="53" t="str">
-        <x:v>廠商</x:v>
-      </x:c>
-      <x:c r="E33" s="57" t="str">
-        <x:v>示範廠商 A</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="34" customHeight="1">
-      <x:c r="A34" s="52" t="str">
-        <x:v>Sourcing Status</x:v>
-      </x:c>
-      <x:c r="B34" s="52" t="str">
-        <x:v>CE 從來源帶出</x:v>
-      </x:c>
-      <x:c r="C34" s="53" t="str">
-        <x:v>保留公司／原廠供應與核准狀態原文，例如 Approved、Active、NRND、Obsolete；不得用它取代右側零件狀態。</x:v>
-      </x:c>
-      <x:c r="D34" s="53" t="str">
-        <x:v>供應／核准狀態</x:v>
-      </x:c>
-      <x:c r="E34" s="57" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="34" customHeight="1">
-      <x:c r="A35" s="52" t="str">
-        <x:v>Virtual PN</x:v>
-      </x:c>
-      <x:c r="B35" s="52" t="str">
-        <x:v>CE 從來源帶出</x:v>
-      </x:c>
-      <x:c r="C35" s="53" t="str">
-        <x:v>來源有值才帶出；無值留白，不要自編 TX。</x:v>
-      </x:c>
-      <x:c r="D35" s="53" t="str">
-        <x:v>TX（第一優先）</x:v>
-      </x:c>
-      <x:c r="E35" s="57" t="str">
-        <x:v>DEMO-TX-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="34" customHeight="1">
-      <x:c r="A36" s="52" t="str">
-        <x:v>PEGA P/N</x:v>
-      </x:c>
-      <x:c r="B36" s="52" t="str">
-        <x:v>CE 從來源帶出</x:v>
-      </x:c>
-      <x:c r="C36" s="53" t="str">
-        <x:v>來源有值才帶出；Virtual PN 空白時才作為 TX 後備值，無值留白。</x:v>
-      </x:c>
-      <x:c r="D36" s="53" t="str">
-        <x:v>TX（第二優先）</x:v>
-      </x:c>
-      <x:c r="E36" s="57" t="str">
-        <x:v>DEMO-PEGA-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="34" customHeight="1">
-      <x:c r="A37" s="52" t="str">
-        <x:v>Ref_tmp</x:v>
-      </x:c>
-      <x:c r="B37" s="52" t="str">
-        <x:v>原始分組／CE 保留</x:v>
-      </x:c>
-      <x:c r="C37" s="53" t="str">
-        <x:v>可留白由工具依 Ref Des 分組；本範本若填寫，使用與 Ref Des 相同的完整位號集合，同組替代料相鄰排列。</x:v>
-      </x:c>
-      <x:c r="D37" s="53" t="str">
-        <x:v>Ref Group</x:v>
-      </x:c>
-      <x:c r="E37" s="57" t="str">
-        <x:v>C101, C102</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="34" customHeight="1">
-      <x:c r="A38" s="52" t="str">
-        <x:v>LV</x:v>
-      </x:c>
-      <x:c r="B38" s="52" t="str">
-        <x:v>來源資料／CE 保留</x:v>
-      </x:c>
-      <x:c r="C38" s="53" t="str">
-        <x:v>來源有版次就保留，不另造版本。</x:v>
-      </x:c>
-      <x:c r="D38" s="53" t="str">
-        <x:v>版次</x:v>
-      </x:c>
-      <x:c r="E38" s="57" t="str">
-        <x:v>A</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="34" customHeight="1">
-      <x:c r="A39" s="52" t="str">
-        <x:v>CIS/Remark</x:v>
-      </x:c>
-      <x:c r="B39" s="52" t="str">
-        <x:v>來源參考／CE 保留</x:v>
-      </x:c>
-      <x:c r="C39" s="53" t="str">
-        <x:v>只供原 Excel 參考；網站不匯入此欄，也不把它當成 RD 追蹤說明。</x:v>
-      </x:c>
-      <x:c r="D39" s="53" t="str">
-        <x:v>不匯入</x:v>
-      </x:c>
-      <x:c r="E39" s="57" t="str">
-        <x:v>來源備註（選填）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="34" customHeight="1">
-      <x:c r="A40" s="52" t="str">
-        <x:v>Part Number</x:v>
-      </x:c>
-      <x:c r="B40" s="52" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="C40" s="53" t="str">
-        <x:v>填公司正式料號並保留前導零；查無時留白，於零件狀態填待確認，不把廠商 MPN／TX 填進這欄。</x:v>
-      </x:c>
-      <x:c r="D40" s="53" t="str">
-        <x:v>內部料號</x:v>
-      </x:c>
-      <x:c r="E40" s="57" t="str">
-        <x:v>000-DEMO-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="34" customHeight="1">
-      <x:c r="A41" s="52" t="str">
-        <x:v>Part Name</x:v>
-      </x:c>
-      <x:c r="B41" s="52" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="C41" s="53" t="str">
-        <x:v>來源有公司料名就保留；無資料可留白。</x:v>
-      </x:c>
-      <x:c r="D41" s="53" t="str">
-        <x:v>內部料名</x:v>
-      </x:c>
-      <x:c r="E41" s="57" t="str">
-        <x:v>示範電容</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="34" customHeight="1">
-      <x:c r="A42" s="52" t="str">
-        <x:v>Part Spec</x:v>
-      </x:c>
-      <x:c r="B42" s="52" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C42" s="53" t="str">
-        <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
-      </x:c>
-      <x:c r="D42" s="53" t="str">
-        <x:v>規格</x:v>
-      </x:c>
-      <x:c r="E42" s="57" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="34" customHeight="1">
-      <x:c r="A43" s="52" t="str">
-        <x:v>Schematic_Part</x:v>
-      </x:c>
-      <x:c r="B43" s="52" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C43" s="53" t="str">
-        <x:v>原 BOM 有原理圖符號就保留；無資料可留白，不要求 CE 新建符號。</x:v>
-      </x:c>
-      <x:c r="D43" s="53" t="str">
-        <x:v>Symbol</x:v>
-      </x:c>
-      <x:c r="E43" s="57" t="str">
-        <x:v>CAP</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="34" customHeight="1">
-      <x:c r="A44" s="52" t="str">
-        <x:v>PCB_Footprint</x:v>
-      </x:c>
-      <x:c r="B44" s="52" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C44" s="53" t="str">
-        <x:v>原 BOM 有封裝就保留；無資料可留白，不要求 CE 新建封裝。</x:v>
-      </x:c>
-      <x:c r="D44" s="53" t="str">
-        <x:v>Footprint</x:v>
-      </x:c>
-      <x:c r="E44" s="57" t="str">
-        <x:v>C_0402</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="34" customHeight="1">
-      <x:c r="A45" s="54" t="str">
-        <x:v>零件狀態</x:v>
-      </x:c>
-      <x:c r="B45" s="54" t="str">
-        <x:v>CE 補欄／帶出原文</x:v>
-      </x:c>
-      <x:c r="C45" s="55" t="str">
-        <x:v>本次交付必須補在最右側。填公司新設計使用限制原文；不明填待確認，供 RD 後續確認與參考。</x:v>
-      </x:c>
-      <x:c r="D45" s="55" t="str">
-        <x:v>零件狀態（獨立顯示）</x:v>
-      </x:c>
-      <x:c r="E45" s="58" t="str">
-        <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>